<commit_message>
Updates to misfiled and missing sheets
</commit_message>
<xml_diff>
--- a/LOCATION-SHEETS/MISSING-SHEETS.xlsx
+++ b/LOCATION-SHEETS/MISSING-SHEETS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11113"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ed/Documents/GitHub/rainfall-rescue/LOCATION-SHEETS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owner\Git\Rainfall\DQ_Checks\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A531EDB6-A328-6946-B6CD-67B77AC1098C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73D59FF1-B6D0-4853-AF04-BFF491AF4CDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="1660" windowWidth="27200" windowHeight="14880" xr2:uid="{BBF0E115-4142-CB48-B420-5D0EBD0E64F7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BBF0E115-4142-CB48-B420-5D0EBD0E64F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="91">
   <si>
     <t>Station name</t>
   </si>
@@ -211,6 +211,102 @@
   </si>
   <si>
     <t>TOMINTOUL</t>
+  </si>
+  <si>
+    <t>Braemar Canmore</t>
+  </si>
+  <si>
+    <t>County</t>
+  </si>
+  <si>
+    <t>Aberdeenshire</t>
+  </si>
+  <si>
+    <t>[Leftover]</t>
+  </si>
+  <si>
+    <t>Clackmannanshire</t>
+  </si>
+  <si>
+    <t>Derbyshire</t>
+  </si>
+  <si>
+    <t>Hertfordshire</t>
+  </si>
+  <si>
+    <t>Banffshire</t>
+  </si>
+  <si>
+    <t>Shropshire</t>
+  </si>
+  <si>
+    <t>Berkshire</t>
+  </si>
+  <si>
+    <t>Cumberland</t>
+  </si>
+  <si>
+    <t>Brecknockshire</t>
+  </si>
+  <si>
+    <t>Yorkshire West Riding</t>
+  </si>
+  <si>
+    <t>Nottinghamshire</t>
+  </si>
+  <si>
+    <t>Middlesex</t>
+  </si>
+  <si>
+    <t>Yorkshire North Riding</t>
+  </si>
+  <si>
+    <t>Lincolnshire</t>
+  </si>
+  <si>
+    <t>Essex</t>
+  </si>
+  <si>
+    <t>Radnorshire</t>
+  </si>
+  <si>
+    <t>Yorkshire East Riding</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>BR has Days of Rain ?</t>
+  </si>
+  <si>
+    <t>Lanarkshire</t>
+  </si>
+  <si>
+    <t>5163/9</t>
+  </si>
+  <si>
+    <t>Crawford - Camps Reservoir - Linnburn</t>
+  </si>
+  <si>
+    <t>Holy Loch Rosmor</t>
+  </si>
+  <si>
+    <t>Argyll</t>
+  </si>
+  <si>
+    <t>PARKHILL-FILTERS-PORT-GLASGOW-WW</t>
+  </si>
+  <si>
+    <t>Renfrewshire</t>
+  </si>
+  <si>
+    <t>Parkhill Filters - Port Glasgow WW</t>
+  </si>
+  <si>
+    <t>5309</t>
   </si>
 </sst>
 </file>
@@ -260,20 +356,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -295,9 +390,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -335,7 +430,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -441,7 +536,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -583,7 +678,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -591,396 +686,608 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC75AAC6-CB18-4040-A1AE-A5995A9D3845}">
-  <dimension ref="A1:E33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="35.5" style="2" customWidth="1"/>
-    <col min="3" max="3" width="28.5" style="6" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="2"/>
+    <col min="1" max="1" width="42.625" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="28.5" style="5" customWidth="1"/>
+    <col min="4" max="4" width="22.625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="19.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>1840</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="E2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>1860</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+      <c r="E3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>1860</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="E4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>1870</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="E5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>1870</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+      <c r="E6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>1880</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="E7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>1880</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+      <c r="E8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1880</v>
+      </c>
+      <c r="E9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C10" s="5">
         <v>2309</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D10" s="3">
         <v>1890</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="E10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C11" s="5">
         <v>804</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D11" s="3">
         <v>1900</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+      <c r="E11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C12" s="5">
         <v>2667</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D12" s="3">
         <v>1910</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+      <c r="E12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C13" s="5">
         <v>3626</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D13" s="3">
         <v>1910</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+      <c r="E13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D14" s="3">
         <v>1910</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+      <c r="E14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B15" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D15" s="3">
         <v>1910</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+      <c r="E15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B16" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D16" s="3">
         <v>1910</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+      <c r="E16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B17" t="s">
         <v>50</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D17" s="3">
         <v>1910</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+      <c r="E17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="3">
+        <v>1910</v>
+      </c>
+      <c r="E18" t="s">
+        <v>61</v>
+      </c>
+      <c r="F18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B19" t="s">
         <v>43</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C19" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D19" s="3">
         <v>1920</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+      <c r="E19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B20" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C20" s="5">
         <v>2651</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D20" s="3">
         <v>1920</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+      <c r="E20" t="s">
+        <v>64</v>
+      </c>
+      <c r="F20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B21" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C21" s="5">
         <v>890</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D21" s="3">
         <v>1920</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+      <c r="E21" t="s">
+        <v>73</v>
+      </c>
+      <c r="F21" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B22" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C22" s="5">
         <v>3468</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D22" s="3">
         <v>1920</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
+      <c r="E22" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B23" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C23" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D23" s="3">
         <v>1920</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
+      <c r="E23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F23" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B24" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C24" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D24" s="3">
         <v>1920</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
+      <c r="E24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D25" s="3">
+        <v>1920</v>
+      </c>
+      <c r="E25" t="s">
+        <v>88</v>
+      </c>
+      <c r="F25" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B26" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C26" s="5">
         <v>4227</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D26" s="3">
         <v>1930</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" ht="19" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+      <c r="E26" t="s">
+        <v>77</v>
+      </c>
+      <c r="F26" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B27" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D27" s="3">
         <v>1930</v>
       </c>
-      <c r="E24" s="7"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
+      <c r="E27" t="s">
+        <v>74</v>
+      </c>
+      <c r="F27" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B28" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C28" s="5">
         <v>3407</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D28" s="3">
         <v>1930</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
+      <c r="E28" t="s">
+        <v>78</v>
+      </c>
+      <c r="F28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B29" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D29" s="3">
         <v>1950</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" ht="19" x14ac:dyDescent="0.2">
-      <c r="A30" s="7"/>
-    </row>
-    <row r="31" spans="1:5" ht="19" x14ac:dyDescent="0.2">
-      <c r="A31" s="7"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32"/>
-    </row>
-    <row r="33" spans="1:1" ht="19" x14ac:dyDescent="0.2">
-      <c r="A33" s="7"/>
+      <c r="E29" t="s">
+        <v>75</v>
+      </c>
+      <c r="F29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>84</v>
+      </c>
+      <c r="B30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D30" s="3">
+        <v>1950</v>
+      </c>
+      <c r="E30" t="s">
+        <v>82</v>
+      </c>
+      <c r="F30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="6"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D26">
-    <sortCondition ref="D2:D26"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D29">
+    <sortCondition ref="D2:D29"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>